<commit_message>
Recuperacion de funcionalidad Modal Detected 19 ITEM
</commit_message>
<xml_diff>
--- a/app/database/MRA11/mroy_MRA1_09_Diaphragm_Rupture.xlsx
+++ b/app/database/MRA11/mroy_MRA1_09_Diaphragm_Rupture.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
   <si>
     <t xml:space="preserve">code</t>
   </si>
@@ -43,6 +43,18 @@
     <t xml:space="preserve">notes</t>
   </si>
   <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None (Standard)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All plunger codes and liquid ends </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No rupture detection system</t>
+  </si>
+  <si>
     <t xml:space="preserve">Direct Attach Head Mounted Pressure type with gauge only</t>
   </si>
   <si>
@@ -70,49 +82,13 @@
     <t xml:space="preserve">Pressure type with gauge and Ex Proof Switch</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Double diaphragm with intermediate fluid. N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">o probe. Not available on plunger codes C</t>
-    </r>
+    <t xml:space="preserve">Double diaphragm with intermediate fluid. No probe. Not available on plunger codes C</t>
   </si>
   <si>
     <t xml:space="preserve"> D and H</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Double diaphragm with intermediate fluid and probe. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Not available on plunger codes C</t>
-    </r>
+    <t xml:space="preserve">Double diaphragm with intermediate fluid and probe. Not available on plunger codes C</t>
   </si>
 </sst>
 </file>
@@ -203,7 +179,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -213,6 +189,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -440,18 +436,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1048576"/>
+  <dimension ref="A1:AK1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="54.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="55.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="8" style="1" width="10.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="15" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="8" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -477,205 +472,268 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="n">
+    <row r="2" s="7" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="6"/>
+      <c r="Z2" s="6"/>
+      <c r="AA2" s="6"/>
+      <c r="AB2" s="6"/>
+      <c r="AC2" s="6"/>
+      <c r="AD2" s="6"/>
+      <c r="AE2" s="6"/>
+      <c r="AF2" s="6"/>
+      <c r="AG2" s="6"/>
+      <c r="AH2" s="6"/>
+      <c r="AI2" s="6"/>
+      <c r="AJ2" s="6"/>
+      <c r="AK2" s="6"/>
+    </row>
+    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>1921</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>2721</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>3464</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>4117</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>986</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>1921</v>
-      </c>
-      <c r="F2" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>2721</v>
-      </c>
-      <c r="F3" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="B8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>3076</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>3464</v>
-      </c>
-      <c r="F4" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>4117</v>
-      </c>
-      <c r="F5" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>986</v>
-      </c>
-      <c r="F6" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-    </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>3076</v>
-      </c>
-      <c r="F7" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="L7" s="0"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="7"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="7"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="7"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="G12" s="7"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="G13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-    </row>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+    </row>
     <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>